<commit_message>
SWBM SFR file handling
</commit_message>
<xml_diff>
--- a/SWBM_Test/SWBM_Test_questions.xlsx
+++ b/SWBM_Test/SWBM_Test_questions.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20391"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D93417D-9299-4CCA-8432-A47013C07672}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A295762-7253-45DA-86E8-4CD3C483AB02}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Questions" sheetId="1" r:id="rId1"/>
@@ -13,6 +13,7 @@
     <sheet name="Changes, Gus22 to new SWBM" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
   <si>
     <t>filename</t>
   </si>
@@ -91,6 +92,15 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>SFR_subws_flows_partitioning.txt</t>
+  </si>
+  <si>
+    <t>How is this file generated?</t>
+  </si>
+  <si>
+    <t>Also does this file ever get used?</t>
   </si>
 </sst>
 </file>
@@ -409,13 +419,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -426,12 +436,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>